<commit_message>
Update Supplementary Figures 7 and 12 source data
Correct TRL classifications for ThorCon 500 (1 to 3) and Thorizon (4 to 1), consistent with Kang et al. (2026).

Replace the source-data workbooks for Supplementary Figures 7 and 12 with their revised versions.
</commit_message>
<xml_diff>
--- a/revision/data/Supplementary/sfig07_source_data_vendors_trl.xlsx
+++ b/revision/data/Supplementary/sfig07_source_data_vendors_trl.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79f001dfc2d9feea/Nature_Energy_SMRs_2026/Extended Data/Extended_Data_Files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79f001dfc2d9feea/Nat. Comms v2/Supplementary source data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{62286390-28C3-43A4-AC5D-D38473C632BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3571A39B-7E2E-475F-9E10-A3494610F42A}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{62286390-28C3-43A4-AC5D-D38473C632BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A24AD333-EA92-4E76-A123-007F5837AA9A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0A382E72-BA5E-4CC8-9797-B43F3A36ADD4}"/>
   </bookViews>
@@ -288,7 +288,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -300,6 +300,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -325,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -335,6 +342,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -674,7 +684,7 @@
   <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" customWidth="1"/>
     <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -724,81 +734,81 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B2" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="D2" s="2">
-        <v>2027.2697237518919</v>
+        <v>2038.6797550154099</v>
       </c>
       <c r="E2" s="2">
-        <v>2026.303454989765</v>
+        <v>2034.461640517417</v>
       </c>
       <c r="F2" s="4">
-        <v>2026</v>
+        <v>2030</v>
       </c>
       <c r="G2" s="4">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K2" s="4">
-        <v>125</v>
+        <v>55</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="4">
-        <v>6</v>
+        <v>56</v>
+      </c>
+      <c r="B3" s="5">
+        <v>3</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D3" s="2">
-        <v>2027.27394271048</v>
+        <v>2041.697924838548</v>
       </c>
       <c r="E3" s="2">
-        <v>2026.309891834371</v>
+        <v>2035.484288290095</v>
       </c>
       <c r="F3" s="4">
-        <v>2026</v>
+        <v>2032</v>
       </c>
       <c r="G3" s="4">
+        <v>15</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="4">
+        <v>500</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="4">
-        <v>300</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>22</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>17</v>
@@ -806,163 +816,163 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="B4" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2">
-        <v>2029.3204685672431</v>
+        <v>2043.459643151047</v>
       </c>
       <c r="E4" s="2">
-        <v>2028.1689750891931</v>
+        <v>2037.7864832332971</v>
       </c>
       <c r="F4" s="4">
-        <v>2028</v>
+        <v>2031.9</v>
       </c>
       <c r="G4" s="4">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K4" s="4">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="B5" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="D5" s="2">
-        <v>2032.1316914378549</v>
+        <v>2045.437657412107</v>
       </c>
       <c r="E5" s="2">
-        <v>2029.9430492742661</v>
+        <v>2039.1844390703709</v>
       </c>
       <c r="F5" s="4">
-        <v>2029.9</v>
+        <v>2035</v>
       </c>
       <c r="G5" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K5" s="4">
-        <v>300</v>
+        <v>168</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="B6" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="D6" s="2">
-        <v>2033.1194121230531</v>
+        <v>2046.2504131832629</v>
       </c>
       <c r="E6" s="2">
-        <v>2030.958929558185</v>
+        <v>2038.7714461414939</v>
       </c>
       <c r="F6" s="4">
-        <v>2030</v>
+        <v>2034</v>
       </c>
       <c r="G6" s="4">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="4">
+        <v>60</v>
+      </c>
+      <c r="L6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="4">
-        <v>82.5</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="M6" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="B7" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D7" s="2">
-        <v>2033.4577557182611</v>
+        <v>2046.7201725512321</v>
       </c>
       <c r="E7" s="2">
-        <v>2030.9518977604171</v>
+        <v>2039.592962564144</v>
       </c>
       <c r="F7" s="4">
-        <v>2029</v>
+        <v>2033</v>
       </c>
       <c r="G7" s="4">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K7" s="4">
         <v>100</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>17</v>
@@ -970,37 +980,37 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="B8" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="D8" s="2">
-        <v>2035.109373018744</v>
+        <v>2046.9739035148191</v>
       </c>
       <c r="E8" s="2">
-        <v>2032.9426184350591</v>
+        <v>2039.8330228895741</v>
       </c>
       <c r="F8" s="4">
-        <v>2031</v>
+        <v>2035</v>
       </c>
       <c r="G8" s="4">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K8" s="4">
-        <v>107</v>
+        <v>400</v>
       </c>
       <c r="L8" s="4" t="s">
         <v>12</v>
@@ -1011,25 +1021,25 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="B9" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="D9" s="2">
-        <v>2035.118749466382</v>
+        <v>2047.0917141291261</v>
       </c>
       <c r="E9" s="2">
-        <v>2032.962125294222</v>
+        <v>2040.0536816682879</v>
       </c>
       <c r="F9" s="4">
-        <v>2033</v>
+        <v>2036</v>
       </c>
       <c r="G9" s="4">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>25</v>
@@ -1041,36 +1051,36 @@
         <v>18</v>
       </c>
       <c r="K9" s="4">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B10" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D10" s="2">
-        <v>2036.8511575215359</v>
+        <v>2047.237119490725</v>
       </c>
       <c r="E10" s="2">
-        <v>2032.2631584409</v>
+        <v>2040.016849369088</v>
       </c>
       <c r="F10" s="4">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="G10" s="4">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>25</v>
@@ -1082,80 +1092,80 @@
         <v>18</v>
       </c>
       <c r="K10" s="4">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="B11" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D11" s="2">
-        <v>2036.8798923115421</v>
+        <v>2048.1435725766328</v>
       </c>
       <c r="E11" s="2">
-        <v>2032.266231890924</v>
+        <v>2040.8700655997859</v>
       </c>
       <c r="F11" s="4">
         <v>2033</v>
       </c>
       <c r="G11" s="4">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K11" s="4">
-        <v>195</v>
+        <v>55</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="B12" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D12" s="2">
-        <v>2037.040162758341</v>
+        <v>2048.7537021238309</v>
       </c>
       <c r="E12" s="2">
-        <v>2032.691616859141</v>
+        <v>2041.65800297178</v>
       </c>
       <c r="F12" s="4">
-        <v>2032.5</v>
+        <v>2034</v>
       </c>
       <c r="G12" s="4">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>30</v>
@@ -1164,39 +1174,39 @@
         <v>18</v>
       </c>
       <c r="K12" s="4">
-        <v>470</v>
+        <v>300</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="B13" s="4">
         <v>1</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D13" s="2">
-        <v>2038.6797550154099</v>
+        <v>2048.7914736183379</v>
       </c>
       <c r="E13" s="2">
-        <v>2034.461640517417</v>
+        <v>2041.656349056007</v>
       </c>
       <c r="F13" s="4">
-        <v>2030</v>
+        <v>2035</v>
       </c>
       <c r="G13" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>30</v>
@@ -1205,7 +1215,7 @@
         <v>18</v>
       </c>
       <c r="K13" s="4">
-        <v>55</v>
+        <v>150</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>22</v>
@@ -1216,37 +1226,37 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B14" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D14" s="2">
-        <v>2038.6995708996401</v>
+        <v>2048.8172093316698</v>
       </c>
       <c r="E14" s="2">
-        <v>2034.4667334848359</v>
+        <v>2041.6492241567371</v>
       </c>
       <c r="F14" s="4">
-        <v>2031.7</v>
+        <v>2034</v>
       </c>
       <c r="G14" s="4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K14" s="4">
-        <v>345</v>
+        <v>110</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>22</v>
@@ -1257,37 +1267,37 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B15" s="4">
         <v>1</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D15" s="2">
-        <v>2041.697924838548</v>
+        <v>2048.822538340451</v>
       </c>
       <c r="E15" s="2">
-        <v>2035.484288290095</v>
+        <v>2041.6409863053359</v>
       </c>
       <c r="F15" s="4">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="G15" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J15" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K15" s="4">
-        <v>500</v>
+        <v>110</v>
       </c>
       <c r="L15" s="4" t="s">
         <v>31</v>
@@ -1298,66 +1308,66 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B16" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D16" s="2">
-        <v>2042.1038663939919</v>
+        <v>2049.7984378851152</v>
       </c>
       <c r="E16" s="2">
-        <v>2035.926336243152</v>
+        <v>2042.634057638872</v>
       </c>
       <c r="F16" s="4">
-        <v>2033.5</v>
+        <v>2035</v>
       </c>
       <c r="G16" s="4">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J16" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K16" s="4">
-        <v>300</v>
+        <v>50</v>
       </c>
       <c r="L16" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>23</v>
+        <v>67</v>
       </c>
       <c r="B17" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="2">
-        <v>2042.1491981498441</v>
+        <v>2042.1038663939919</v>
       </c>
       <c r="E17" s="2">
-        <v>2036.2577518337041</v>
+        <v>2035.926336243152</v>
       </c>
       <c r="F17" s="4">
-        <v>2028</v>
+        <v>2033.5</v>
       </c>
       <c r="G17" s="4">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>25</v>
@@ -1369,133 +1379,133 @@
         <v>18</v>
       </c>
       <c r="K17" s="4">
-        <v>75</v>
+        <v>300</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="B18" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D18" s="2">
-        <v>2042.186375821329</v>
+        <v>2043.4449015239391</v>
       </c>
       <c r="E18" s="2">
-        <v>2036.2381773369441</v>
+        <v>2037.7697615323141</v>
       </c>
       <c r="F18" s="4">
-        <v>2029</v>
+        <v>2033</v>
       </c>
       <c r="G18" s="4">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K18" s="4">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="B19" s="4">
         <v>2</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D19" s="2">
-        <v>2043.4449015239391</v>
+        <v>2047.4136090597981</v>
       </c>
       <c r="E19" s="2">
-        <v>2037.7697615323141</v>
+        <v>2040.2037780255639</v>
       </c>
       <c r="F19" s="4">
-        <v>2033</v>
+        <v>2030</v>
       </c>
       <c r="G19" s="4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K19" s="4">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="L19" s="4" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="M19" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B20" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="D20" s="2">
-        <v>2043.459643151047</v>
+        <v>2033.1194121230531</v>
       </c>
       <c r="E20" s="2">
-        <v>2037.7864832332971</v>
+        <v>2030.958929558185</v>
       </c>
       <c r="F20" s="4">
-        <v>2031.9</v>
+        <v>2030</v>
       </c>
       <c r="G20" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J20" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K20" s="4">
-        <v>200</v>
+        <v>82.5</v>
       </c>
       <c r="L20" s="4" t="s">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="M20" s="4" t="s">
         <v>17</v>
@@ -1503,119 +1513,119 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="B21" s="4">
         <v>3</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="D21" s="2">
-        <v>2043.488533649499</v>
+        <v>2033.4577557182611</v>
       </c>
       <c r="E21" s="2">
-        <v>2037.752914005097</v>
+        <v>2030.9518977604171</v>
       </c>
       <c r="F21" s="4">
-        <v>2033</v>
+        <v>2029</v>
       </c>
       <c r="G21" s="4">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K21" s="4">
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="L21" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M21" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="B22" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D22" s="2">
-        <v>2045.437657412107</v>
+        <v>2036.8511575215359</v>
       </c>
       <c r="E22" s="2">
-        <v>2039.1844390703709</v>
+        <v>2032.2631584409</v>
       </c>
       <c r="F22" s="4">
-        <v>2035</v>
+        <v>2030</v>
       </c>
       <c r="G22" s="4">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K22" s="4">
-        <v>168</v>
+        <v>300</v>
       </c>
       <c r="L22" s="4" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="B23" s="4">
         <v>3</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D23" s="2">
-        <v>2046.1552113377411</v>
+        <v>2036.8798923115421</v>
       </c>
       <c r="E23" s="2">
-        <v>2038.73915128968</v>
+        <v>2032.266231890924</v>
       </c>
       <c r="F23" s="4">
-        <v>2028</v>
+        <v>2033</v>
       </c>
       <c r="G23" s="4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J23" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K23" s="4">
-        <v>42</v>
+        <v>195</v>
       </c>
       <c r="L23" s="4" t="s">
         <v>31</v>
@@ -1626,37 +1636,37 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="B24" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D24" s="2">
-        <v>2046.2504131832629</v>
+        <v>2037.040162758341</v>
       </c>
       <c r="E24" s="2">
-        <v>2038.7714461414939</v>
+        <v>2032.691616859141</v>
       </c>
       <c r="F24" s="4">
-        <v>2034</v>
+        <v>2032.5</v>
       </c>
       <c r="G24" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="J24" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K24" s="4">
-        <v>60</v>
+        <v>470</v>
       </c>
       <c r="L24" s="4" t="s">
         <v>12</v>
@@ -1667,40 +1677,40 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B25" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D25" s="2">
-        <v>2046.7201725512321</v>
+        <v>2038.6995708996401</v>
       </c>
       <c r="E25" s="2">
-        <v>2039.592962564144</v>
+        <v>2034.4667334848359</v>
       </c>
       <c r="F25" s="4">
-        <v>2033</v>
+        <v>2031.7</v>
       </c>
       <c r="G25" s="4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J25" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K25" s="4">
-        <v>100</v>
+        <v>345</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="M25" s="4" t="s">
         <v>17</v>
@@ -1708,69 +1718,69 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="B26" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D26" s="2">
-        <v>2046.9739035148191</v>
+        <v>2042.1491981498441</v>
       </c>
       <c r="E26" s="2">
-        <v>2039.8330228895741</v>
+        <v>2036.2577518337041</v>
       </c>
       <c r="F26" s="4">
-        <v>2035</v>
+        <v>2028</v>
       </c>
       <c r="G26" s="4">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J26" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K26" s="4">
-        <v>400</v>
+        <v>75</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="B27" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D27" s="2">
-        <v>2047.0917141291261</v>
+        <v>2042.186375821329</v>
       </c>
       <c r="E27" s="2">
-        <v>2040.0536816682879</v>
+        <v>2036.2381773369441</v>
       </c>
       <c r="F27" s="4">
-        <v>2036</v>
+        <v>2029</v>
       </c>
       <c r="G27" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>26</v>
@@ -1779,10 +1789,10 @@
         <v>18</v>
       </c>
       <c r="K27" s="4">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="M27" s="4" t="s">
         <v>17</v>
@@ -1790,78 +1800,78 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B28" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D28" s="2">
-        <v>2047.174916888943</v>
+        <v>2043.488533649499</v>
       </c>
       <c r="E28" s="2">
-        <v>2040.0131142393709</v>
+        <v>2037.752914005097</v>
       </c>
       <c r="F28" s="4">
         <v>2033</v>
       </c>
       <c r="G28" s="4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K28" s="4">
-        <v>100</v>
+        <v>170</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="M28" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B29" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D29" s="2">
-        <v>2047.237119490725</v>
+        <v>2046.1552113377411</v>
       </c>
       <c r="E29" s="2">
-        <v>2040.016849369088</v>
+        <v>2038.73915128968</v>
       </c>
       <c r="F29" s="4">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="G29" s="4">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J29" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K29" s="4">
-        <v>100</v>
+        <v>42</v>
       </c>
       <c r="L29" s="4" t="s">
         <v>31</v>
@@ -1872,78 +1882,78 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B30" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D30" s="2">
-        <v>2047.4136090597981</v>
+        <v>2035.109373018744</v>
       </c>
       <c r="E30" s="2">
-        <v>2040.2037780255639</v>
+        <v>2032.9426184350591</v>
       </c>
       <c r="F30" s="4">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="G30" s="4">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="J30" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K30" s="4">
-        <v>40</v>
+        <v>107</v>
       </c>
       <c r="L30" s="4" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="M30" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="B31" s="4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D31" s="2">
-        <v>2048.1435725766328</v>
+        <v>2035.118749466382</v>
       </c>
       <c r="E31" s="2">
-        <v>2040.8700655997859</v>
+        <v>2032.962125294222</v>
       </c>
       <c r="F31" s="4">
         <v>2033</v>
       </c>
       <c r="G31" s="4">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="H31" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J31" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K31" s="4">
         <v>77</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J31" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K31" s="4">
-        <v>55</v>
       </c>
       <c r="L31" s="4" t="s">
         <v>12</v>
@@ -1953,29 +1963,29 @@
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" s="4">
+      <c r="A32" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B32" s="5">
         <v>1</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>28</v>
       </c>
       <c r="D32" s="2">
-        <v>2048.7537021238309</v>
+        <v>2047.174916888943</v>
       </c>
       <c r="E32" s="2">
-        <v>2041.65800297178</v>
+        <v>2040.0131142393709</v>
       </c>
       <c r="F32" s="4">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="G32" s="4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="I32" s="4" t="s">
         <v>30</v>
@@ -1984,10 +1994,10 @@
         <v>18</v>
       </c>
       <c r="K32" s="4">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="M32" s="4" t="s">
         <v>17</v>
@@ -1995,78 +2005,78 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="B33" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D33" s="2">
-        <v>2048.7914736183379</v>
+        <v>2027.2697237518919</v>
       </c>
       <c r="E33" s="2">
-        <v>2041.656349056007</v>
+        <v>2026.303454989765</v>
       </c>
       <c r="F33" s="4">
-        <v>2035</v>
+        <v>2026</v>
       </c>
       <c r="G33" s="4">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K33" s="4">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="L33" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="M33" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="B34" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D34" s="2">
-        <v>2048.8172093316698</v>
+        <v>2027.27394271048</v>
       </c>
       <c r="E34" s="2">
-        <v>2041.6492241567371</v>
+        <v>2026.309891834371</v>
       </c>
       <c r="F34" s="4">
-        <v>2034</v>
+        <v>2026</v>
       </c>
       <c r="G34" s="4">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="J34" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="K34" s="4">
-        <v>110</v>
+        <v>300</v>
       </c>
       <c r="L34" s="4" t="s">
         <v>22</v>
@@ -2077,84 +2087,84 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="B35" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D35" s="2">
-        <v>2048.822538340451</v>
+        <v>2029.3204685672431</v>
       </c>
       <c r="E35" s="2">
-        <v>2041.6409863053359</v>
+        <v>2028.1689750891931</v>
       </c>
       <c r="F35" s="4">
-        <v>2033</v>
+        <v>2028</v>
       </c>
       <c r="G35" s="4">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="I35" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="K35" s="4">
         <v>30</v>
       </c>
-      <c r="J35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K35" s="4">
-        <v>110</v>
-      </c>
       <c r="L35" s="4" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="M35" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="B36" s="4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D36" s="2">
-        <v>2049.7984378851152</v>
+        <v>2032.1316914378549</v>
       </c>
       <c r="E36" s="2">
-        <v>2042.634057638872</v>
+        <v>2029.9430492742661</v>
       </c>
       <c r="F36" s="4">
-        <v>2035</v>
+        <v>2029.9</v>
       </c>
       <c r="G36" s="4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J36" s="4" t="s">
         <v>18</v>
       </c>
       <c r="K36" s="4">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="L36" s="4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="M36" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
@@ -2164,7 +2174,7 @@
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M38">
-    <sortCondition ref="D1:D38"/>
+    <sortCondition ref="B1:B38"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>